<commit_message>
update many stuff: write easy-reading RX & Copay dataframes, delete unnecessary chunks and files, run test w/ age_cat
</commit_message>
<xml_diff>
--- a/test results_strength n quantity.xlsx
+++ b/test results_strength n quantity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/liley/Documents/Smith/Special Study w: Rob/IQVIA21_SQL/IQVIA21_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{199054A9-4A76-F542-82FE-51294DB463F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5983A796-CABA-2941-B413-A9A56FFED5E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1940" yWindow="740" windowWidth="27460" windowHeight="16760" activeTab="1" xr2:uid="{7D789166-7FD4-FF4E-9E05-0DAA6FD18114}"/>
+    <workbookView xWindow="11580" yWindow="3740" windowWidth="16120" windowHeight="16720" activeTab="3" xr2:uid="{7D789166-7FD4-FF4E-9E05-0DAA6FD18114}"/>
   </bookViews>
   <sheets>
     <sheet name="strength_NY" sheetId="2" r:id="rId1"/>
@@ -2630,6 +2630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10666F38-8901-0443-8989-34426375F3A8}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
@@ -2697,7 +2698,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" hidden="1">
       <c r="A3" s="1" t="s">
         <v>97</v>
       </c>
@@ -2718,7 +2719,7 @@
         <v>0.99750000000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" hidden="1">
       <c r="A4" s="1" t="s">
         <v>98</v>
       </c>
@@ -2739,7 +2740,7 @@
         <v>0.99209999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" hidden="1">
       <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
@@ -2788,7 +2789,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" hidden="1">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -2921,7 +2922,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" hidden="1">
       <c r="A12" s="1" t="s">
         <v>93</v>
       </c>
@@ -2942,7 +2943,7 @@
         <v>0.99460000000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" hidden="1">
       <c r="A13" s="1" t="s">
         <v>94</v>
       </c>
@@ -2963,7 +2964,7 @@
         <v>0.94650000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" hidden="1">
       <c r="A14" s="1" t="s">
         <v>95</v>
       </c>
@@ -3012,7 +3013,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" hidden="1">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -3033,7 +3034,7 @@
         <v>0.69620000000000004</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" hidden="1">
       <c r="A17" s="1" t="s">
         <v>23</v>
       </c>
@@ -3082,7 +3083,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" hidden="1">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -3131,7 +3132,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" hidden="1">
       <c r="A21" s="1" t="s">
         <v>54</v>
       </c>
@@ -3180,7 +3181,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" hidden="1">
       <c r="A23" s="1" t="s">
         <v>65</v>
       </c>
@@ -3313,7 +3314,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" hidden="1">
       <c r="A28" s="1" t="s">
         <v>75</v>
       </c>
@@ -3334,7 +3335,7 @@
         <v>0.34760000000000002</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" hidden="1">
       <c r="A29" s="1" t="s">
         <v>77</v>
       </c>
@@ -3355,7 +3356,7 @@
         <v>0.69489999999999996</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" hidden="1">
       <c r="A30" s="1" t="s">
         <v>79</v>
       </c>
@@ -3544,7 +3545,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" hidden="1">
       <c r="A37" s="1" t="s">
         <v>91</v>
       </c>
@@ -3565,7 +3566,7 @@
         <v>0.99680000000000002</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" hidden="1">
       <c r="A38" s="1" t="s">
         <v>92</v>
       </c>
@@ -3586,7 +3587,7 @@
         <v>0.99760000000000004</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" hidden="1">
       <c r="A39" s="1" t="s">
         <v>96</v>
       </c>
@@ -3607,7 +3608,7 @@
         <v>0.98240000000000005</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" hidden="1">
       <c r="A40" s="1" t="s">
         <v>101</v>
       </c>
@@ -3628,7 +3629,7 @@
         <v>7.8200000000000006E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" hidden="1">
       <c r="A41" s="1" t="s">
         <v>19</v>
       </c>
@@ -3649,7 +3650,7 @@
         <v>0.67049999999999998</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" hidden="1">
       <c r="A42" s="1" t="s">
         <v>22</v>
       </c>
@@ -3670,7 +3671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" hidden="1">
       <c r="A43" s="1" t="s">
         <v>24</v>
       </c>
@@ -3691,7 +3692,7 @@
         <v>0.28570000000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" hidden="1">
       <c r="A44" s="1" t="s">
         <v>25</v>
       </c>
@@ -3712,7 +3713,7 @@
         <v>0.99690000000000001</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" hidden="1">
       <c r="A45" s="1" t="s">
         <v>27</v>
       </c>
@@ -3733,7 +3734,7 @@
         <v>0.99480000000000002</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" hidden="1">
       <c r="A46" s="1" t="s">
         <v>28</v>
       </c>
@@ -3754,7 +3755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" hidden="1">
       <c r="A47" s="1" t="s">
         <v>29</v>
       </c>
@@ -3775,7 +3776,7 @@
         <v>0.77839999999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" hidden="1">
       <c r="A48" s="1" t="s">
         <v>30</v>
       </c>
@@ -3796,7 +3797,7 @@
         <v>0.26679999999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" hidden="1">
       <c r="A49" s="1" t="s">
         <v>32</v>
       </c>
@@ -3817,7 +3818,7 @@
         <v>0.99809999999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" hidden="1">
       <c r="A50" s="1" t="s">
         <v>33</v>
       </c>
@@ -3838,7 +3839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" hidden="1">
       <c r="A51" s="1" t="s">
         <v>34</v>
       </c>
@@ -3859,7 +3860,7 @@
         <v>0.4027</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" hidden="1">
       <c r="A52" s="1" t="s">
         <v>35</v>
       </c>
@@ -3880,7 +3881,7 @@
         <v>0.85929999999999995</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" hidden="1">
       <c r="A53" s="1" t="s">
         <v>37</v>
       </c>
@@ -3901,7 +3902,7 @@
         <v>0.84740000000000004</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" hidden="1">
       <c r="A54" s="1" t="s">
         <v>38</v>
       </c>
@@ -3922,7 +3923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" hidden="1">
       <c r="A55" s="1" t="s">
         <v>39</v>
       </c>
@@ -3943,7 +3944,7 @@
         <v>0.47320000000000001</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" hidden="1">
       <c r="A56" s="11" t="s">
         <v>40</v>
       </c>
@@ -3964,7 +3965,7 @@
         <v>0.1827</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" hidden="1">
       <c r="A57" s="1" t="s">
         <v>41</v>
       </c>
@@ -3985,7 +3986,7 @@
         <v>0.74419999999999997</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" hidden="1">
       <c r="A58" s="1" t="s">
         <v>42</v>
       </c>
@@ -4006,7 +4007,7 @@
         <v>0.88360000000000005</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" hidden="1">
       <c r="A59" s="1" t="s">
         <v>43</v>
       </c>
@@ -4027,7 +4028,7 @@
         <v>0.68700000000000006</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" hidden="1">
       <c r="A60" s="1" t="s">
         <v>44</v>
       </c>
@@ -4048,7 +4049,7 @@
         <v>0.51200000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" hidden="1">
       <c r="A61" s="1" t="s">
         <v>45</v>
       </c>
@@ -4069,7 +4070,7 @@
         <v>0.55130000000000001</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" hidden="1">
       <c r="A62" s="1" t="s">
         <v>46</v>
       </c>
@@ -4090,7 +4091,7 @@
         <v>0.23730000000000001</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" hidden="1">
       <c r="A63" s="1" t="s">
         <v>47</v>
       </c>
@@ -4111,7 +4112,7 @@
         <v>0.29820000000000002</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" hidden="1">
       <c r="A64" s="1" t="s">
         <v>48</v>
       </c>
@@ -4132,7 +4133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" hidden="1">
       <c r="A65" s="1" t="s">
         <v>50</v>
       </c>
@@ -4153,7 +4154,7 @@
         <v>0.68030000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" hidden="1">
       <c r="A66" s="1" t="s">
         <v>51</v>
       </c>
@@ -4174,7 +4175,7 @@
         <v>0.12709999999999999</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" hidden="1">
       <c r="A67" s="11" t="s">
         <v>52</v>
       </c>
@@ -4195,7 +4196,7 @@
         <v>0.94220000000000004</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" hidden="1">
       <c r="A68" s="1" t="s">
         <v>53</v>
       </c>
@@ -4216,7 +4217,7 @@
         <v>0.63690000000000002</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" hidden="1">
       <c r="A69" s="11" t="s">
         <v>55</v>
       </c>
@@ -4237,7 +4238,7 @@
         <v>0.83640000000000003</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" hidden="1">
       <c r="A70" s="11" t="s">
         <v>56</v>
       </c>
@@ -4258,7 +4259,7 @@
         <v>0.2016</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" hidden="1">
       <c r="A71" s="1" t="s">
         <v>57</v>
       </c>
@@ -4279,7 +4280,7 @@
         <v>0.47560000000000002</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" hidden="1">
       <c r="A72" s="11" t="s">
         <v>58</v>
       </c>
@@ -4300,7 +4301,7 @@
         <v>0.68830000000000002</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" hidden="1">
       <c r="A73" s="1" t="s">
         <v>59</v>
       </c>
@@ -4321,7 +4322,7 @@
         <v>0.25159999999999999</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" hidden="1">
       <c r="A74" s="1" t="s">
         <v>61</v>
       </c>
@@ -4342,7 +4343,7 @@
         <v>0.60850000000000004</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" hidden="1">
       <c r="A75" s="1" t="s">
         <v>62</v>
       </c>
@@ -4363,7 +4364,7 @@
         <v>0.86960000000000004</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" hidden="1">
       <c r="A76" s="11" t="s">
         <v>63</v>
       </c>
@@ -4384,7 +4385,7 @@
         <v>0.53620000000000001</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" hidden="1">
       <c r="A77" s="1" t="s">
         <v>64</v>
       </c>
@@ -4405,7 +4406,7 @@
         <v>0.51349999999999996</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" hidden="1">
       <c r="A78" s="1" t="s">
         <v>66</v>
       </c>
@@ -4426,7 +4427,7 @@
         <v>0.93530000000000002</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" hidden="1">
       <c r="A79" s="1" t="s">
         <v>68</v>
       </c>
@@ -4447,7 +4448,7 @@
         <v>0.3997</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" hidden="1">
       <c r="A80" s="11" t="s">
         <v>69</v>
       </c>
@@ -4468,7 +4469,7 @@
         <v>0.51390000000000002</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" hidden="1">
       <c r="A81" s="11" t="s">
         <v>71</v>
       </c>
@@ -4489,7 +4490,7 @@
         <v>0.97599999999999998</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" hidden="1">
       <c r="A82" s="1" t="s">
         <v>73</v>
       </c>
@@ -4510,7 +4511,7 @@
         <v>0.6704</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" hidden="1">
       <c r="A83" s="11" t="s">
         <v>76</v>
       </c>
@@ -4531,7 +4532,7 @@
         <v>0.70050000000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" hidden="1">
       <c r="A84" s="1" t="s">
         <v>78</v>
       </c>
@@ -4552,7 +4553,7 @@
         <v>0.32129999999999997</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" hidden="1">
       <c r="A85" s="1" t="s">
         <v>80</v>
       </c>
@@ -4573,7 +4574,7 @@
         <v>0.96099999999999997</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" hidden="1">
       <c r="A86" s="11" t="s">
         <v>81</v>
       </c>
@@ -4594,7 +4595,7 @@
         <v>0.12939999999999999</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" hidden="1">
       <c r="A87" s="1" t="s">
         <v>82</v>
       </c>
@@ -4615,7 +4616,7 @@
         <v>0.98519999999999996</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" hidden="1">
       <c r="A88" s="1" t="s">
         <v>83</v>
       </c>
@@ -4636,7 +4637,7 @@
         <v>0.22539999999999999</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" hidden="1">
       <c r="A89" s="1" t="s">
         <v>84</v>
       </c>
@@ -4657,7 +4658,7 @@
         <v>0.99970000000000003</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" hidden="1">
       <c r="A90" s="1" t="s">
         <v>85</v>
       </c>
@@ -4678,7 +4679,7 @@
         <v>0.89380000000000004</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" hidden="1">
       <c r="A91" s="1" t="s">
         <v>86</v>
       </c>
@@ -4699,7 +4700,7 @@
         <v>0.75849999999999995</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" hidden="1">
       <c r="A92" s="1" t="s">
         <v>88</v>
       </c>
@@ -4720,7 +4721,7 @@
         <v>0.20039999999999999</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" hidden="1">
       <c r="A93" s="1" t="s">
         <v>89</v>
       </c>
@@ -4741,7 +4742,7 @@
         <v>0.99870000000000003</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" hidden="1">
       <c r="A94" s="1" t="s">
         <v>4</v>
       </c>
@@ -4762,7 +4763,7 @@
         <v>0.9748</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" hidden="1">
       <c r="A95" s="1" t="s">
         <v>5</v>
       </c>
@@ -4783,7 +4784,7 @@
         <v>0.97070000000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" hidden="1">
       <c r="A96" s="1" t="s">
         <v>10</v>
       </c>
@@ -4804,7 +4805,7 @@
         <v>5.9900000000000002E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" hidden="1">
       <c r="A97" s="1" t="s">
         <v>13</v>
       </c>
@@ -4825,7 +4826,7 @@
         <v>0.97909999999999997</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" hidden="1">
       <c r="A98" s="1" t="s">
         <v>15</v>
       </c>
@@ -4833,7 +4834,7 @@
         <v>-21.85</v>
       </c>
       <c r="C98" s="12">
-        <f t="shared" ref="C98:C129" si="4">EXP(B98)</f>
+        <f t="shared" ref="C98" si="4">EXP(B98)</f>
         <v>3.240899549293071E-10</v>
       </c>
       <c r="D98" s="12">
@@ -4847,7 +4848,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H98" xr:uid="{10666F38-8901-0443-8989-34426375F3A8}"/>
+  <autoFilter ref="A1:H98" xr:uid="{10666F38-8901-0443-8989-34426375F3A8}">
+    <filterColumn colId="6">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H98">
     <sortCondition descending="1" ref="H2:H98"/>
   </sortState>
@@ -7960,7 +7967,7 @@
         <v>45.07</v>
       </c>
       <c r="C2" s="14">
-        <f>EXP(B2)</f>
+        <f t="shared" ref="C2:C33" si="0">EXP(B2)</f>
         <v>3.7467291515305165E+19</v>
       </c>
       <c r="D2" s="14">
@@ -7981,7 +7988,7 @@
         <v>44.71</v>
       </c>
       <c r="C3" s="14">
-        <f>EXP(B3)</f>
+        <f t="shared" si="0"/>
         <v>2.6140042292230435E+19</v>
       </c>
       <c r="D3" s="14">
@@ -8002,7 +8009,7 @@
         <v>25.99</v>
       </c>
       <c r="C4" s="14">
-        <f>EXP(B4)</f>
+        <f t="shared" si="0"/>
         <v>193782067274.81113</v>
       </c>
       <c r="D4" s="14">
@@ -8023,7 +8030,7 @@
         <v>19.55</v>
       </c>
       <c r="C5" s="14">
-        <f>EXP(B5)</f>
+        <f t="shared" si="0"/>
         <v>309354986.78036124</v>
       </c>
       <c r="D5" s="14">
@@ -8044,7 +8051,7 @@
         <v>17.88</v>
       </c>
       <c r="C6" s="14">
-        <f>EXP(B6)</f>
+        <f t="shared" si="0"/>
         <v>58235168.502116203</v>
       </c>
       <c r="D6" s="14">
@@ -8065,7 +8072,7 @@
         <v>7.5720000000000001</v>
       </c>
       <c r="C7" s="14">
-        <f>EXP(B7)</f>
+        <f t="shared" si="0"/>
         <v>1943.0224429892489</v>
       </c>
       <c r="D7" s="14">
@@ -8093,7 +8100,7 @@
         <v>5.5419999999999998</v>
       </c>
       <c r="C8" s="14">
-        <f>EXP(B8)</f>
+        <f t="shared" si="0"/>
         <v>255.18786515321113</v>
       </c>
       <c r="D8" s="14">
@@ -8121,7 +8128,7 @@
         <v>2.4870000000000001</v>
       </c>
       <c r="C9" s="14">
-        <f>EXP(B9)</f>
+        <f t="shared" si="0"/>
         <v>12.025146513590867</v>
       </c>
       <c r="D9" s="14">
@@ -8145,7 +8152,7 @@
         <v>2.4550000000000001</v>
       </c>
       <c r="C10" s="14">
-        <f>EXP(B10)</f>
+        <f t="shared" si="0"/>
         <v>11.646433548879468</v>
       </c>
       <c r="D10" s="14">
@@ -8173,7 +8180,7 @@
         <v>2.19</v>
       </c>
       <c r="C11" s="14">
-        <f>EXP(B11)</f>
+        <f t="shared" si="0"/>
         <v>8.9352131146987475</v>
       </c>
       <c r="D11" s="14">
@@ -8194,7 +8201,7 @@
         <v>1.9670000000000001</v>
       </c>
       <c r="C12" s="14">
-        <f>EXP(B12)</f>
+        <f t="shared" si="0"/>
         <v>7.1491966946819137</v>
       </c>
       <c r="D12" s="14">
@@ -8222,7 +8229,7 @@
         <v>1.925</v>
       </c>
       <c r="C13" s="14">
-        <f>EXP(B13)</f>
+        <f t="shared" si="0"/>
         <v>6.8551486658991783</v>
       </c>
       <c r="D13" s="14">
@@ -8246,7 +8253,7 @@
         <v>1.8660000000000001</v>
       </c>
       <c r="C14" s="14">
-        <f>EXP(B14)</f>
+        <f t="shared" si="0"/>
         <v>6.4623950509214172</v>
       </c>
       <c r="D14" s="14">
@@ -8267,7 +8274,7 @@
         <v>1.6910000000000001</v>
       </c>
       <c r="C15" s="14">
-        <f>EXP(B15)</f>
+        <f t="shared" si="0"/>
         <v>5.4249028964801633</v>
       </c>
       <c r="D15" s="14">
@@ -8288,7 +8295,7 @@
         <v>1.216</v>
       </c>
       <c r="C16" s="14">
-        <f>EXP(B16)</f>
+        <f t="shared" si="0"/>
         <v>3.3736660440948167</v>
       </c>
       <c r="D16" s="14">
@@ -8316,7 +8323,7 @@
         <v>0.97760000000000002</v>
       </c>
       <c r="C17" s="14">
-        <f>EXP(B17)</f>
+        <f t="shared" si="0"/>
         <v>2.6580692144475377</v>
       </c>
       <c r="D17" s="14">
@@ -8337,7 +8344,7 @@
         <v>0.79510000000000003</v>
       </c>
       <c r="C18" s="14">
-        <f>EXP(B18)</f>
+        <f t="shared" si="0"/>
         <v>2.2146624519763289</v>
       </c>
       <c r="D18" s="14">
@@ -8365,7 +8372,7 @@
         <v>0.73650000000000004</v>
       </c>
       <c r="C19" s="14">
-        <f>EXP(B19)</f>
+        <f t="shared" si="0"/>
         <v>2.0886125628345509</v>
       </c>
       <c r="D19" s="14">
@@ -8386,7 +8393,7 @@
         <v>0.70740000000000003</v>
       </c>
       <c r="C20" s="14">
-        <f>EXP(B20)</f>
+        <f t="shared" si="0"/>
         <v>2.0287097503103557</v>
       </c>
       <c r="D20" s="14">
@@ -8407,7 +8414,7 @@
         <v>0.42420000000000002</v>
       </c>
       <c r="C21" s="14">
-        <f>EXP(B21)</f>
+        <f t="shared" si="0"/>
         <v>1.5283672366660834</v>
       </c>
       <c r="D21" s="14">
@@ -8428,7 +8435,7 @@
         <v>0.41189999999999999</v>
       </c>
       <c r="C22" s="14">
-        <f>EXP(B22)</f>
+        <f t="shared" si="0"/>
         <v>1.5096834604340326</v>
       </c>
       <c r="D22" s="14">
@@ -8449,7 +8456,7 @@
         <v>0.39489999999999997</v>
       </c>
       <c r="C23" s="14">
-        <f>EXP(B23)</f>
+        <f t="shared" si="0"/>
         <v>1.4842357599234954</v>
       </c>
       <c r="D23" s="14">
@@ -8470,7 +8477,7 @@
         <v>0.34739999999999999</v>
       </c>
       <c r="C24" s="14">
-        <f>EXP(B24)</f>
+        <f t="shared" si="0"/>
         <v>1.4153827652610078</v>
       </c>
       <c r="D24" s="14">
@@ -8491,7 +8498,7 @@
         <v>0.31</v>
       </c>
       <c r="C25" s="14">
-        <f>EXP(B25)</f>
+        <f t="shared" si="0"/>
         <v>1.3634251141321778</v>
       </c>
       <c r="D25" s="14">
@@ -8512,7 +8519,7 @@
         <v>0.30570000000000003</v>
       </c>
       <c r="C26" s="14">
-        <f>EXP(B26)</f>
+        <f t="shared" si="0"/>
         <v>1.3575749729590214</v>
       </c>
       <c r="D26" s="14">
@@ -8533,7 +8540,7 @@
         <v>0.29620000000000002</v>
       </c>
       <c r="C27" s="14">
-        <f>EXP(B27)</f>
+        <f t="shared" si="0"/>
         <v>1.3447390777546151</v>
       </c>
       <c r="D27" s="14">
@@ -8554,7 +8561,7 @@
         <v>0.28920000000000001</v>
       </c>
       <c r="C28" s="14">
-        <f>EXP(B28)</f>
+        <f t="shared" si="0"/>
         <v>1.335358773577829</v>
       </c>
       <c r="D28" s="14">
@@ -8575,7 +8582,7 @@
         <v>0.27739999999999998</v>
       </c>
       <c r="C29" s="14">
-        <f>EXP(B29)</f>
+        <f t="shared" si="0"/>
         <v>1.3196941431307549</v>
       </c>
       <c r="D29" s="14">
@@ -8596,7 +8603,7 @@
         <v>0.2737</v>
       </c>
       <c r="C30" s="14">
-        <f>EXP(B30)</f>
+        <f t="shared" si="0"/>
         <v>1.314820296976801</v>
       </c>
       <c r="D30" s="14">
@@ -8617,7 +8624,7 @@
         <v>0.2238</v>
       </c>
       <c r="C31" s="14">
-        <f>EXP(B31)</f>
+        <f t="shared" si="0"/>
         <v>1.250820830244229</v>
       </c>
       <c r="D31" s="14">
@@ -8642,7 +8649,7 @@
         <v>0.2225</v>
       </c>
       <c r="C32" s="14">
-        <f>EXP(B32)</f>
+        <f t="shared" si="0"/>
         <v>1.249195819650653</v>
       </c>
       <c r="D32" s="14">
@@ -8663,7 +8670,7 @@
         <v>0.21260000000000001</v>
       </c>
       <c r="C33" s="14">
-        <f>EXP(B33)</f>
+        <f t="shared" si="0"/>
         <v>1.236889796360678</v>
       </c>
       <c r="D33" s="14">
@@ -8684,7 +8691,7 @@
         <v>0.21240000000000001</v>
       </c>
       <c r="C34" s="14">
-        <f>EXP(B34)</f>
+        <f t="shared" ref="C34:C65" si="1">EXP(B34)</f>
         <v>1.2366424431375527</v>
       </c>
       <c r="D34" s="14">
@@ -8705,7 +8712,7 @@
         <v>0.2089</v>
       </c>
       <c r="C35" s="14">
-        <f>EXP(B35)</f>
+        <f t="shared" si="1"/>
         <v>1.2323217601924215</v>
       </c>
       <c r="D35" s="14">
@@ -8726,7 +8733,7 @@
         <v>0.20660000000000001</v>
       </c>
       <c r="C36" s="14">
-        <f>EXP(B36)</f>
+        <f t="shared" si="1"/>
         <v>1.2294906771375276</v>
       </c>
       <c r="D36" s="14">
@@ -8747,7 +8754,7 @@
         <v>0.18540000000000001</v>
       </c>
       <c r="C37" s="14">
-        <f>EXP(B37)</f>
+        <f t="shared" si="1"/>
         <v>1.2036998237740573</v>
       </c>
       <c r="D37" s="14">
@@ -8768,7 +8775,7 @@
         <v>0.1648</v>
       </c>
       <c r="C38" s="14">
-        <f>EXP(B38)</f>
+        <f t="shared" si="1"/>
         <v>1.1791572636739382</v>
       </c>
       <c r="D38" s="14">
@@ -8789,7 +8796,7 @@
         <v>0.13980000000000001</v>
       </c>
       <c r="C39" s="14">
-        <f>EXP(B39)</f>
+        <f t="shared" si="1"/>
         <v>1.1500437671013981</v>
       </c>
       <c r="D39" s="14">
@@ -8810,7 +8817,7 @@
         <v>0.13850000000000001</v>
       </c>
       <c r="C40" s="14">
-        <f>EXP(B40)</f>
+        <f t="shared" si="1"/>
         <v>1.1485496815701788</v>
       </c>
       <c r="D40" s="14">
@@ -8831,7 +8838,7 @@
         <v>0.1144</v>
       </c>
       <c r="C41" s="14">
-        <f>EXP(B41)</f>
+        <f t="shared" si="1"/>
         <v>1.1212005154062326</v>
       </c>
       <c r="D41" s="14">
@@ -8852,7 +8859,7 @@
         <v>0.1076</v>
       </c>
       <c r="C42" s="14">
-        <f>EXP(B42)</f>
+        <f t="shared" si="1"/>
         <v>1.1136022154002507</v>
       </c>
       <c r="D42" s="14">
@@ -8873,7 +8880,7 @@
         <v>9.3399999999999997E-2</v>
       </c>
       <c r="C43" s="14">
-        <f>EXP(B43)</f>
+        <f t="shared" si="1"/>
         <v>1.0979008077708354</v>
       </c>
       <c r="D43" s="14">
@@ -8894,7 +8901,7 @@
         <v>9.2490000000000003E-2</v>
       </c>
       <c r="C44" s="14">
-        <f>EXP(B44)</f>
+        <f t="shared" si="1"/>
         <v>1.0969021724837338</v>
       </c>
       <c r="D44" s="14">
@@ -8915,7 +8922,7 @@
         <v>7.9829999999999998E-2</v>
       </c>
       <c r="C45" s="14">
-        <f>EXP(B45)</f>
+        <f t="shared" si="1"/>
         <v>1.083102924526065</v>
       </c>
       <c r="D45" s="14">
@@ -8936,7 +8943,7 @@
         <v>7.6340000000000005E-2</v>
       </c>
       <c r="C46" s="14">
-        <f>EXP(B46)</f>
+        <f t="shared" si="1"/>
         <v>1.0793294838036027</v>
       </c>
       <c r="D46" s="14">
@@ -8957,7 +8964,7 @@
         <v>7.3469999999999994E-2</v>
       </c>
       <c r="C47" s="14">
-        <f>EXP(B47)</f>
+        <f t="shared" si="1"/>
         <v>1.0762362491001076</v>
       </c>
       <c r="D47" s="14">
@@ -8978,7 +8985,7 @@
         <v>6.4329999999999998E-2</v>
       </c>
       <c r="C48" s="14">
-        <f>EXP(B48)</f>
+        <f t="shared" si="1"/>
         <v>1.0664442673082135</v>
       </c>
       <c r="D48" s="14">
@@ -8999,7 +9006,7 @@
         <v>3.6130000000000002E-2</v>
       </c>
       <c r="C49" s="14">
-        <f>EXP(B49)</f>
+        <f t="shared" si="1"/>
         <v>1.0367906205110891</v>
       </c>
       <c r="D49" s="14">
@@ -9020,7 +9027,7 @@
         <v>3.524E-2</v>
       </c>
       <c r="C50" s="14">
-        <f>EXP(B50)</f>
+        <f t="shared" si="1"/>
         <v>1.035868287357969</v>
       </c>
       <c r="D50" s="14">
@@ -9038,7 +9045,7 @@
         <v>132</v>
       </c>
       <c r="C51" s="14">
-        <f>EXP(B51)</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="H51" s="2" t="str">
@@ -9054,7 +9061,7 @@
         <v>-3.8630000000000001E-3</v>
       </c>
       <c r="C52" s="14">
-        <f>EXP(B52)</f>
+        <f t="shared" si="1"/>
         <v>0.99614445178599542</v>
       </c>
       <c r="D52" s="14">
@@ -9078,7 +9085,7 @@
         <v>-4.1310000000000001E-3</v>
       </c>
       <c r="C53" s="14">
-        <f>EXP(B53)</f>
+        <f t="shared" si="1"/>
         <v>0.99587752084326076</v>
       </c>
       <c r="D53" s="14">
@@ -9103,7 +9110,7 @@
         <v>-7.2449999999999997E-3</v>
       </c>
       <c r="C54" s="14">
-        <f>EXP(B54)</f>
+        <f t="shared" si="1"/>
         <v>0.99278118174542873</v>
       </c>
       <c r="D54" s="14">
@@ -9124,7 +9131,7 @@
         <v>-1.8069999999999999E-2</v>
       </c>
       <c r="C55" s="14">
-        <f>EXP(B55)</f>
+        <f t="shared" si="1"/>
         <v>0.98209228349227407</v>
       </c>
       <c r="D55" s="14">
@@ -9145,7 +9152,7 @@
         <v>-2.0109999999999999E-2</v>
       </c>
       <c r="C56" s="14">
-        <f>EXP(B56)</f>
+        <f t="shared" si="1"/>
         <v>0.98009085738267609</v>
       </c>
       <c r="D56" s="14">
@@ -9166,7 +9173,7 @@
         <v>-2.342E-2</v>
       </c>
       <c r="C57" s="14">
-        <f>EXP(B57)</f>
+        <f t="shared" si="1"/>
         <v>0.97685211971257735</v>
       </c>
       <c r="D57" s="14">
@@ -9187,7 +9194,7 @@
         <v>-3.7679999999999998E-2</v>
       </c>
       <c r="C58" s="14">
-        <f>EXP(B58)</f>
+        <f t="shared" si="1"/>
         <v>0.96302105832844542</v>
       </c>
       <c r="D58" s="14">
@@ -9208,7 +9215,7 @@
         <v>-4.2560000000000001E-2</v>
       </c>
       <c r="C59" s="14">
-        <f>EXP(B59)</f>
+        <f t="shared" si="1"/>
         <v>0.95833296381808397</v>
       </c>
       <c r="D59" s="14">
@@ -9229,7 +9236,7 @@
         <v>-9.0840000000000004E-2</v>
       </c>
       <c r="C60" s="14">
-        <f>EXP(B60)</f>
+        <f t="shared" si="1"/>
         <v>0.91316380542025966</v>
       </c>
       <c r="D60" s="14">
@@ -9250,7 +9257,7 @@
         <v>-0.1115</v>
       </c>
       <c r="C61" s="14">
-        <f>EXP(B61)</f>
+        <f t="shared" si="1"/>
         <v>0.89449139140326783</v>
       </c>
       <c r="D61" s="14">
@@ -9271,7 +9278,7 @@
         <v>-0.1376</v>
       </c>
       <c r="C62" s="14">
-        <f>EXP(B62)</f>
+        <f t="shared" si="1"/>
         <v>0.87144720091968464</v>
       </c>
       <c r="D62" s="14">
@@ -9292,7 +9299,7 @@
         <v>-0.13880000000000001</v>
       </c>
       <c r="C63" s="14">
-        <f>EXP(B63)</f>
+        <f t="shared" si="1"/>
         <v>0.87040209146966419</v>
       </c>
       <c r="D63" s="14">
@@ -9313,7 +9320,7 @@
         <v>-0.21590000000000001</v>
       </c>
       <c r="C64" s="14">
-        <f>EXP(B64)</f>
+        <f t="shared" si="1"/>
         <v>0.80581587943247779</v>
       </c>
       <c r="D64" s="14">
@@ -9334,7 +9341,7 @@
         <v>-0.23719999999999999</v>
       </c>
       <c r="C65" s="14">
-        <f>EXP(B65)</f>
+        <f t="shared" si="1"/>
         <v>0.78883350553878007</v>
       </c>
       <c r="D65" s="14">
@@ -9355,7 +9362,7 @@
         <v>-0.2581</v>
       </c>
       <c r="C66" s="14">
-        <f>EXP(B66)</f>
+        <f t="shared" ref="C66:C97" si="2">EXP(B66)</f>
         <v>0.77251797644656472</v>
       </c>
       <c r="D66" s="14">
@@ -9376,7 +9383,7 @@
         <v>-0.27550000000000002</v>
       </c>
       <c r="C67" s="14">
-        <f>EXP(B67)</f>
+        <f t="shared" si="2"/>
         <v>0.75919243209404896</v>
       </c>
       <c r="D67" s="14">
@@ -9397,7 +9404,7 @@
         <v>-0.31259999999999999</v>
       </c>
       <c r="C68" s="14">
-        <f>EXP(B68)</f>
+        <f t="shared" si="2"/>
         <v>0.73154247104170333</v>
       </c>
       <c r="D68" s="14">
@@ -9418,7 +9425,7 @@
         <v>-0.3271</v>
       </c>
       <c r="C69" s="14">
-        <f>EXP(B69)</f>
+        <f t="shared" si="2"/>
         <v>0.72101163825760284</v>
       </c>
       <c r="D69" s="14">
@@ -9439,7 +9446,7 @@
         <v>-0.37290000000000001</v>
       </c>
       <c r="C70" s="14">
-        <f>EXP(B70)</f>
+        <f t="shared" si="2"/>
         <v>0.68873410281068115</v>
       </c>
       <c r="D70" s="14">
@@ -9460,7 +9467,7 @@
         <v>-0.51519999999999999</v>
       </c>
       <c r="C71" s="14">
-        <f>EXP(B71)</f>
+        <f t="shared" si="2"/>
         <v>0.59738110644852915</v>
       </c>
       <c r="D71" s="14">
@@ -9481,7 +9488,7 @@
         <v>-0.61550000000000005</v>
       </c>
       <c r="C72" s="14">
-        <f>EXP(B72)</f>
+        <f t="shared" si="2"/>
         <v>0.54037064243051181</v>
       </c>
       <c r="D72" s="14">
@@ -9502,7 +9509,7 @@
         <v>-0.69810000000000005</v>
       </c>
       <c r="C73" s="14">
-        <f>EXP(B73)</f>
+        <f t="shared" si="2"/>
         <v>0.49752971277303604</v>
       </c>
       <c r="D73" s="14">
@@ -9526,7 +9533,7 @@
         <v>-0.83160000000000001</v>
       </c>
       <c r="C74" s="14">
-        <f>EXP(B74)</f>
+        <f t="shared" si="2"/>
         <v>0.43535216530895032</v>
       </c>
       <c r="D74" s="14">
@@ -9547,7 +9554,7 @@
         <v>-0.998</v>
       </c>
       <c r="C75" s="14">
-        <f>EXP(B75)</f>
+        <f t="shared" si="2"/>
         <v>0.36861593630341882</v>
       </c>
       <c r="D75" s="14">
@@ -9571,7 +9578,7 @@
         <v>-1.0489999999999999</v>
       </c>
       <c r="C76" s="14">
-        <f>EXP(B76)</f>
+        <f t="shared" si="2"/>
         <v>0.35028786188747862</v>
       </c>
       <c r="D76" s="14">
@@ -9595,7 +9602,7 @@
         <v>-1.149</v>
       </c>
       <c r="C77" s="14">
-        <f>EXP(B77)</f>
+        <f t="shared" si="2"/>
         <v>0.31695356451960294</v>
       </c>
       <c r="D77" s="14">
@@ -9616,7 +9623,7 @@
         <v>-1.1579999999999999</v>
       </c>
       <c r="C78" s="14">
-        <f>EXP(B78)</f>
+        <f t="shared" si="2"/>
         <v>0.31411378063492296</v>
       </c>
       <c r="D78" s="14">
@@ -9632,7 +9639,7 @@
         <v>103</v>
       </c>
       <c r="H78" s="2" t="str">
-        <f>IF(C78&gt;1, "Y", "N")</f>
+        <f t="shared" ref="H78:H86" si="3">IF(C78&gt;1, "Y", "N")</f>
         <v>N</v>
       </c>
     </row>
@@ -9644,7 +9651,7 @@
         <v>-1.335</v>
       </c>
       <c r="C79" s="14">
-        <f>EXP(B79)</f>
+        <f t="shared" si="2"/>
         <v>0.26315817545602871</v>
       </c>
       <c r="D79" s="14">
@@ -9660,7 +9667,7 @@
         <v>103</v>
       </c>
       <c r="H79" s="2" t="str">
-        <f>IF(C79&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9672,7 +9679,7 @@
         <v>-1.4419999999999999</v>
       </c>
       <c r="C80" s="14">
-        <f>EXP(B80)</f>
+        <f t="shared" si="2"/>
         <v>0.2364543767045291</v>
       </c>
       <c r="D80" s="14">
@@ -9688,7 +9695,7 @@
         <v>103</v>
       </c>
       <c r="H80" s="2" t="str">
-        <f>IF(C80&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9700,7 +9707,7 @@
         <v>-1.663</v>
       </c>
       <c r="C81" s="14">
-        <f>EXP(B81)</f>
+        <f t="shared" si="2"/>
         <v>0.18956941793164234</v>
       </c>
       <c r="D81" s="14">
@@ -9716,7 +9723,7 @@
         <v>112</v>
       </c>
       <c r="H81" s="2" t="str">
-        <f>IF(C81&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9728,7 +9735,7 @@
         <v>-3.0459999999999998</v>
       </c>
       <c r="C82" s="14">
-        <f>EXP(B82)</f>
+        <f t="shared" si="2"/>
         <v>4.7548739465768049E-2</v>
       </c>
       <c r="D82" s="14">
@@ -9744,7 +9751,7 @@
         <v>103</v>
       </c>
       <c r="H82" s="2" t="str">
-        <f>IF(C82&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9756,7 +9763,7 @@
         <v>-3.887</v>
       </c>
       <c r="C83" s="14">
-        <f>EXP(B83)</f>
+        <f t="shared" si="2"/>
         <v>2.0506774172181743E-2</v>
       </c>
       <c r="D83" s="14">
@@ -9772,7 +9779,7 @@
         <v>103</v>
       </c>
       <c r="H83" s="2" t="str">
-        <f>IF(C83&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9784,7 +9791,7 @@
         <v>-6.2169999999999996</v>
       </c>
       <c r="C84" s="14">
-        <f>EXP(B84)</f>
+        <f t="shared" si="2"/>
         <v>1.9952219134787581E-3</v>
       </c>
       <c r="D84" s="14">
@@ -9800,7 +9807,7 @@
         <v>103</v>
       </c>
       <c r="H84" s="2" t="str">
-        <f>IF(C84&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9812,7 +9819,7 @@
         <v>-6.673</v>
       </c>
       <c r="C85" s="14">
-        <f>EXP(B85)</f>
+        <f t="shared" si="2"/>
         <v>1.2645992568450805E-3</v>
       </c>
       <c r="D85" s="14">
@@ -9828,7 +9835,7 @@
         <v>103</v>
       </c>
       <c r="H85" s="2" t="str">
-        <f>IF(C85&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9840,7 +9847,7 @@
         <v>-8.0850000000000009</v>
       </c>
       <c r="C86" s="14">
-        <f>EXP(B86)</f>
+        <f t="shared" si="2"/>
         <v>3.0812654468605194E-4</v>
       </c>
       <c r="D86" s="14">
@@ -9856,7 +9863,7 @@
         <v>103</v>
       </c>
       <c r="H86" s="2" t="str">
-        <f>IF(C86&gt;1, "Y", "N")</f>
+        <f t="shared" si="3"/>
         <v>N</v>
       </c>
     </row>
@@ -9868,7 +9875,7 @@
         <v>-12.45</v>
       </c>
       <c r="C87" s="14">
-        <f>EXP(B87)</f>
+        <f t="shared" si="2"/>
         <v>3.9177227660243348E-6</v>
       </c>
       <c r="D87" s="14">
@@ -9889,7 +9896,7 @@
         <v>-14.97</v>
       </c>
       <c r="C88" s="14">
-        <f>EXP(B88)</f>
+        <f t="shared" si="2"/>
         <v>3.1521843310800805E-7</v>
       </c>
       <c r="D88" s="14">
@@ -9910,7 +9917,7 @@
         <v>-15.71</v>
       </c>
       <c r="C89" s="14">
-        <f>EXP(B89)</f>
+        <f t="shared" si="2"/>
         <v>1.5039510086456694E-7</v>
       </c>
       <c r="D89" s="14">
@@ -9931,7 +9938,7 @@
         <v>-20.98</v>
       </c>
       <c r="C90" s="14">
-        <f>EXP(B90)</f>
+        <f t="shared" si="2"/>
         <v>7.7357383093895748E-10</v>
       </c>
       <c r="D90" s="14">
@@ -9952,7 +9959,7 @@
         <v>-21.14</v>
       </c>
       <c r="C91" s="14">
-        <f>EXP(B91)</f>
+        <f t="shared" si="2"/>
         <v>6.5919613534143059E-10</v>
       </c>
       <c r="D91" s="14">
@@ -9973,7 +9980,7 @@
         <v>-21.85</v>
       </c>
       <c r="C92" s="14">
-        <f>EXP(B92)</f>
+        <f t="shared" si="2"/>
         <v>3.240899549293071E-10</v>
       </c>
       <c r="D92" s="14">
@@ -9994,7 +10001,7 @@
         <v>-23.15</v>
       </c>
       <c r="C93" s="14">
-        <f>EXP(B93)</f>
+        <f t="shared" si="2"/>
         <v>8.8324816521196642E-11</v>
       </c>
       <c r="D93" s="14">
@@ -10015,7 +10022,7 @@
         <v>-24.15</v>
       </c>
       <c r="C94" s="14">
-        <f>EXP(B94)</f>
+        <f t="shared" si="2"/>
         <v>3.2492884143387998E-11</v>
       </c>
       <c r="D94" s="14">
@@ -10036,7 +10043,7 @@
         <v>-24.27</v>
       </c>
       <c r="C95" s="14">
-        <f>EXP(B95)</f>
+        <f t="shared" si="2"/>
         <v>2.8818602994653656E-11</v>
       </c>
       <c r="D95" s="14">
@@ -10057,7 +10064,7 @@
         <v>-24.27</v>
       </c>
       <c r="C96" s="14">
-        <f>EXP(B96)</f>
+        <f t="shared" si="2"/>
         <v>2.8818602994653656E-11</v>
       </c>
       <c r="D96" s="14">
@@ -10078,7 +10085,7 @@
         <v>-25.88</v>
       </c>
       <c r="C97" s="14">
-        <f>EXP(B97)</f>
+        <f t="shared" si="2"/>
         <v>5.7604817935801365E-12</v>
       </c>
       <c r="D97" s="14">
@@ -10099,7 +10106,7 @@
         <v>-26.68</v>
       </c>
       <c r="C98" s="14">
-        <f>EXP(B98)</f>
+        <f t="shared" ref="C98:C129" si="4">EXP(B98)</f>
         <v>2.5883513171254756E-12</v>
       </c>
       <c r="D98" s="14">
@@ -10120,7 +10127,7 @@
         <v>-47.86</v>
       </c>
       <c r="C99" s="14">
-        <f>EXP(B99)</f>
+        <f t="shared" si="4"/>
         <v>1.6393289034492922E-21</v>
       </c>
       <c r="D99" s="14">
@@ -10142,6 +10149,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2434E287-2BD6-CC4B-A527-9570EBAD7AAB}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14"/>
   <cols>
@@ -10289,7 +10297,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" hidden="1">
       <c r="A6" s="2" t="s">
         <v>89</v>
       </c>
@@ -10336,7 +10344,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" hidden="1">
       <c r="A8" s="2" t="s">
         <v>84</v>
       </c>
@@ -10383,7 +10391,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" hidden="1">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
@@ -10592,7 +10600,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" hidden="1">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -10612,7 +10620,7 @@
         <v>0.11838</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" hidden="1">
       <c r="A19" s="2" t="s">
         <v>74</v>
       </c>
@@ -10632,7 +10640,7 @@
         <v>0.28860999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" hidden="1">
       <c r="A20" s="2" t="s">
         <v>68</v>
       </c>
@@ -10679,7 +10687,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" hidden="1">
       <c r="A22" s="2" t="s">
         <v>50</v>
       </c>
@@ -10699,7 +10707,7 @@
         <v>0.25368000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" hidden="1">
       <c r="A23" s="2" t="s">
         <v>36</v>
       </c>
@@ -10773,7 +10781,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" hidden="1">
       <c r="A26" s="2" t="s">
         <v>49</v>
       </c>
@@ -10820,7 +10828,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" hidden="1">
       <c r="A28" s="2" t="s">
         <v>54</v>
       </c>
@@ -10867,7 +10875,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" hidden="1">
       <c r="A30" s="2" t="s">
         <v>62</v>
       </c>
@@ -10941,7 +10949,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" hidden="1">
       <c r="A33" s="2" t="s">
         <v>80</v>
       </c>
@@ -10961,7 +10969,7 @@
         <v>0.10703</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" hidden="1">
       <c r="A34" s="2" t="s">
         <v>66</v>
       </c>
@@ -11008,7 +11016,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" hidden="1">
       <c r="A36" s="2" t="s">
         <v>77</v>
       </c>
@@ -11055,7 +11063,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" hidden="1">
       <c r="A38" s="2" t="s">
         <v>73</v>
       </c>
@@ -11075,7 +11083,7 @@
         <v>0.38463999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" hidden="1">
       <c r="A39" s="2" t="s">
         <v>52</v>
       </c>
@@ -11122,7 +11130,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" hidden="1">
       <c r="A41" s="2" t="s">
         <v>71</v>
       </c>
@@ -11142,7 +11150,7 @@
         <v>0.41686000000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" hidden="1">
       <c r="A42" s="2" t="s">
         <v>88</v>
       </c>
@@ -11162,7 +11170,7 @@
         <v>0.44873000000000002</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" hidden="1">
       <c r="A43" s="2" t="s">
         <v>78</v>
       </c>
@@ -11182,7 +11190,7 @@
         <v>0.26274999999999998</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" hidden="1">
       <c r="A44" s="2" t="s">
         <v>23</v>
       </c>
@@ -11202,7 +11210,7 @@
         <v>0.11701</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" hidden="1">
       <c r="A45" s="2" t="s">
         <v>58</v>
       </c>
@@ -11222,7 +11230,7 @@
         <v>0.21704000000000001</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" hidden="1">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
@@ -11242,7 +11250,7 @@
         <v>0.66135999999999995</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" hidden="1">
       <c r="A47" s="2" t="s">
         <v>20</v>
       </c>
@@ -11262,7 +11270,7 @@
         <v>0.24145</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" hidden="1">
       <c r="A48" s="2" t="s">
         <v>59</v>
       </c>
@@ -11282,7 +11290,7 @@
         <v>0.75229000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" hidden="1">
       <c r="A49" s="2" t="s">
         <v>21</v>
       </c>
@@ -11302,7 +11310,7 @@
         <v>0.11527</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" hidden="1">
       <c r="A50" s="2" t="s">
         <v>30</v>
       </c>
@@ -11322,7 +11330,7 @@
         <v>0.17318</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" hidden="1">
       <c r="A51" s="2" t="s">
         <v>56</v>
       </c>
@@ -11342,7 +11350,7 @@
         <v>0.61956999999999995</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" hidden="1">
       <c r="A52" s="2" t="s">
         <v>83</v>
       </c>
@@ -11362,7 +11370,7 @@
         <v>0.47921999999999998</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" hidden="1">
       <c r="A53" s="2" t="s">
         <v>86</v>
       </c>
@@ -11382,7 +11390,7 @@
         <v>0.86907000000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" hidden="1">
       <c r="A54" s="2" t="s">
         <v>82</v>
       </c>
@@ -11429,7 +11437,7 @@
         <v>Y</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" hidden="1">
       <c r="A56" s="2" t="s">
         <v>39</v>
       </c>
@@ -11449,7 +11457,7 @@
         <v>0.98968</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" hidden="1">
       <c r="A57" s="2" t="s">
         <v>37</v>
       </c>
@@ -11469,7 +11477,7 @@
         <v>0.76724999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" hidden="1">
       <c r="A58" s="2" t="s">
         <v>55</v>
       </c>
@@ -11489,7 +11497,7 @@
         <v>0.68103999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" hidden="1">
       <c r="A59" s="2" t="s">
         <v>63</v>
       </c>
@@ -11509,7 +11517,7 @@
         <v>0.77376999999999996</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" hidden="1">
       <c r="A60" s="2" t="s">
         <v>44</v>
       </c>
@@ -11529,7 +11537,7 @@
         <v>0.70216999999999996</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" hidden="1">
       <c r="A61" s="2" t="s">
         <v>29</v>
       </c>
@@ -11549,7 +11557,7 @@
         <v>5.8130000000000001E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" hidden="1">
       <c r="A62" s="2" t="s">
         <v>69</v>
       </c>
@@ -11569,7 +11577,7 @@
         <v>0.19666</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" hidden="1">
       <c r="A63" s="2" t="s">
         <v>79</v>
       </c>
@@ -11589,7 +11597,7 @@
         <v>0.77059999999999995</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" hidden="1">
       <c r="A64" s="2" t="s">
         <v>70</v>
       </c>
@@ -11609,7 +11617,7 @@
         <v>0.68923000000000001</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" hidden="1">
       <c r="A65" s="2" t="s">
         <v>48</v>
       </c>
@@ -11629,7 +11637,7 @@
         <v>0.86585999999999996</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" hidden="1">
       <c r="A66" s="2" t="s">
         <v>35</v>
       </c>
@@ -11649,7 +11657,7 @@
         <v>0.83262000000000003</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" hidden="1">
       <c r="A67" s="2" t="s">
         <v>64</v>
       </c>
@@ -11669,7 +11677,7 @@
         <v>0.31979999999999997</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" hidden="1">
       <c r="A68" s="2" t="s">
         <v>76</v>
       </c>
@@ -11717,7 +11725,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H69" xr:uid="{2434E287-2BD6-CC4B-A527-9570EBAD7AAB}"/>
+  <autoFilter ref="A1:H69" xr:uid="{2434E287-2BD6-CC4B-A527-9570EBAD7AAB}">
+    <filterColumn colId="6">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -20606,7 +20620,7 @@
         <v>0</v>
       </c>
       <c r="E98" s="25">
-        <f t="shared" ref="E98:E129" si="9">SUMIF(B98:D98,"&lt;&gt;#N/A")</f>
+        <f t="shared" ref="E98" si="9">SUMIF(B98:D98,"&lt;&gt;#N/A")</f>
         <v>0</v>
       </c>
       <c r="F98" s="23" t="e">
@@ -20622,11 +20636,11 @@
         <v>#N/A</v>
       </c>
       <c r="J98" s="29">
-        <f t="shared" ref="J98:J129" si="10">SUMIF(F98:I98,"&lt;&gt;#N/A")</f>
+        <f t="shared" ref="J98" si="10">SUMIF(F98:I98,"&lt;&gt;#N/A")</f>
         <v>0</v>
       </c>
       <c r="K98" s="27">
-        <f t="shared" ref="K98:K129" si="11">SUM(E98,J98)</f>
+        <f t="shared" ref="K98" si="11">SUM(E98,J98)</f>
         <v>0</v>
       </c>
       <c r="L98" s="40"/>

</xml_diff>